<commit_message>
Day 3: Storage lifecycle audit, EBS modernisation, and data transfer NAT endpoint remediation
</commit_message>
<xml_diff>
--- a/analysis/savings-model.xlsx
+++ b/analysis/savings-model.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Compute Analysis" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Database Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Storage Analysis" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Data Transfer Analysis" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -154,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -193,6 +196,12 @@
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -586,7 +595,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -623,8 +631,6 @@
         <v>115750</v>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
@@ -960,8 +966,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -969,7 +973,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
         <is>
@@ -1128,7 +1131,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -3768,7 +3770,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4598,4 +4599,1742 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LendFlow Technologies — Storage Estate (S3, EBS, Snapshots) Optimisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Lifecycle Policy Design, GP2 to GP3 Modernisation &amp; Unattached Volume Elimination</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Resource ID / Bucket Name</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Service / Owner</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Capacity (GB)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Current Tier / Type</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Inactivity (Days)</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Current Spend (USD)</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Attachment Status</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Snapshot GB</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Recommended FinOps Action</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>Projected Monthly Savings (USD)</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>Compliance Verification (SOC 2 / RBI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>s3-lendflow-loan-docs-prod</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>s3-bucket</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>kyc-document-service</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>145000</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>S3 Standard</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>180</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>3335</v>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>Apply Lifecycle: &gt;30d to Standard-IA, &gt;90d to Glacier Instant</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>1850</v>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>PCI / SOC 2 WORM Object Lock</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>s3-lendflow-audit-logs-prod</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>s3-bucket</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>platform-compliance</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>85000</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>S3 Standard</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="n">
+        <v>365</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>1955</v>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J6" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>Apply Lifecycle: &gt;90d to Glacier Flexible (SOC 2 / RBI compliant)</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="n">
+        <v>1250</v>
+      </c>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
+          <t>PCI / SOC 2 WORM Object Lock</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>s3-lendflow-raw-analytics-prod</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>s3-bucket</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>analytics-batch-pipeline</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>S3 Standard</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>120</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>2530</v>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J7" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>Enable S3 Intelligent-Tiering for variable analytics data</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>1100</v>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>s3-lendflow-dev-temp-dumps</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>s3-bucket</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>sandbox-experimental</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>S3 Standard</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="n">
+        <v>150</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>805</v>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>Purge temp test dumps &gt;14 days. Apply 14d TTL lifecycle.</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="n">
+        <v>680</v>
+      </c>
+      <c r="M8" s="14" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>vol-0a111111111111111</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>loan-application-service</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>120</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="I9" s="30" t="inlineStr">
+        <is>
+          <t>unattached</t>
+        </is>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>Delete orphaned volume and purge old snapshots</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>vol-0a222222222222222</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>underwriting-engine</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>180</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="I10" s="30" t="inlineStr">
+        <is>
+          <t>unattached</t>
+        </is>
+      </c>
+      <c r="J10" s="28" t="n">
+        <v>2800</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>Delete orphaned volume and purge old snapshots</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>vol-0a333333333333333</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>kyc-document-service</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>90</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>unattached</t>
+        </is>
+      </c>
+      <c r="J11" s="28" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>Delete orphaned volume</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>vol-0a444444444444444</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>perf-testing-load</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>140</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="I12" s="30" t="inlineStr">
+        <is>
+          <t>unattached</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n">
+        <v>3500</v>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>Delete orphaned volume from perf testing</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>vol-0b111111111111111</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>loan-application-service</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>8000</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3 (20% savings + higher baseline IOPS)</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>vol-0b222222222222222</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>underwriting-engine</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G14" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>600</v>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J14" s="29" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3</t>
+        </is>
+      </c>
+      <c r="L14" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="M14" s="14" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>vol-0b333333333333333</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>payment-gateway-service</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J15" s="28" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3 (PCI DSS compliant)</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>vol-0b444444444444444</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>disbursement-engine</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J16" s="29" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3</t>
+        </is>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>60</v>
+      </c>
+      <c r="M16" s="14" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>vol-0b555555555555555</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>analytics-batch-pipeline</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>800</v>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J17" s="28" t="n">
+        <v>18000</v>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3 + purge snapshots &gt;30d</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>160</v>
+      </c>
+      <c r="M17" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>vol-0b666666666666666</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>feature-store-ml</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>prod</t>
+        </is>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <v>500</v>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J18" s="29" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3</t>
+        </is>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>vol-0b777777777777777</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>stage-loan-api</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="E19" s="28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="n">
+        <v>3000</v>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3 &amp; reduce size to 500GB</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="n">
+        <v>130</v>
+      </c>
+      <c r="M19" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>vol-0b888888888888888</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>ebs-volume</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>dev-loan-api</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>gp2</t>
+        </is>
+      </c>
+      <c r="G20" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>Migrate GP2 to GP3 &amp; reduce size to 300GB</t>
+        </is>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>150</v>
+      </c>
+      <c r="M20" s="14" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>snap-fleet-policy-waste</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>ebs-snapshots</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>all-services</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E21" s="28" t="n">
+        <v>65000</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>EBS Snapshot</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>210</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>3250</v>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="J21" s="28" t="n">
+        <v>65000</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>Enforce DLM lifecycle: max 30d retention (saves 50% snapshot spend)</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M21" s="10" t="inlineStr">
+        <is>
+          <t>Standard FinOps cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>17 Storage Assets</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="31">
+        <f>SUM(E5:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="18">
+        <f>SUM(H5:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="17" t="n"/>
+      <c r="J22" s="31">
+        <f>SUM(J5:J21)</f>
+        <v/>
+      </c>
+      <c r="K22" s="17" t="n"/>
+      <c r="L22" s="18">
+        <f>SUM(L5:L21)</f>
+        <v/>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>Achieves $7,600/mo Storage Target</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LendFlow Technologies — Network &amp; Data Transfer Architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Top 10 Costliest Data Transfer Paths, NAT Gateway Bypass &amp; AZ Affinity Remediation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Path ID</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Source Workload &amp; AZ</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Destination Target</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Transfer Classification</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Monthly Volume (GB)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Unit Rate ($/GB)</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Monthly Spend (USD)</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Architectural Root Cause</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Technical Remediation Action</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Compliance Safeguard</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Projected Monthly Savings (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>DT-PATH-01</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>kyc-document-service (ap-south-1a)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>s3-lendflow-loan-docs-prod (via Public NAT)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>NAT Gateway Data Processing</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>105000</v>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>4725</v>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>EC2 downloading S3 docs via Public NAT Gateway instead of S3 Gateway Endpoint</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Deploy AWS S3 Gateway Endpoint (Free route via VPC route table)</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Preserves data localisation and RBI multi-AZ compliance</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>4725</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>DT-PATH-02</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>loan-application-service (ap-south-1a)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>rds-postgres-primary (ap-south-1b)</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Cross-AZ Inter-Service Transfer</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>185000</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>3700</v>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>API in AZ-1a constantly querying Primary DB located in AZ-1b without AZ-affinity</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>Align primary application workloads with DB AZ; use read-replicas in AZ-1a</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>Maintains multi-AZ standby for RBI/SOC2 high availability</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="n">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>DT-PATH-03</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>underwriting-engine (ap-south-1b)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>credit-bureau-connector (ap-south-1c)</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Cross-AZ Inter-Service Transfer</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F7" s="32" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Microservices communicating across AZs through external ALB rather than internal DNS/Service Connect</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Implement AWS Cloud Map / ECS Service Connect with local AZ priority routing</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>Internal TLS 1.3 encryption maintained for PCI DSS</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>DT-PATH-04</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>analytics-batch-pipeline (ap-south-1a)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>s3-lendflow-raw-analytics-prod (via Public NAT)</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>NAT Gateway Data Processing</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F8" s="33" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>Nightly batch ETL downloading large parquet dumps through NAT Gateway</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>Route all S3 analytics traffic through S3 VPC Gateway Endpoint</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>Zero data egress charge via Gateway Endpoint</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>DT-PATH-05</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>api-gateway-mesh (ap-south-1)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>external-client-egress (Internet)</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Internet Egress Transfer</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>80000</v>
+      </c>
+      <c r="F9" s="32" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>7200</v>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Direct API responses, uncompressed JSON payloads, redundant polling headers</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>Enable GZIP/Brotli compression at ALB/CloudFront; implement HTTP 304 caching</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Safe, no compliance breach; improves client latency</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>DT-PATH-06</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>audit-logging-agent (ap-south-1)</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>cloudwatch-logs / datadog (Internet)</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Public NAT / Internet Egress</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F10" s="33" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>1575</v>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Verbose debug logs shipped to external SaaS over NAT Gateway</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>Deploy CloudWatch Logs Interface VPC Endpoint; filter redundant debug logs</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>SOC 2 Type II audit trail fully retained at lower volume</t>
+        </is>
+      </c>
+      <c r="K10" s="15" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>DT-PATH-07</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>payment-gateway-service (ap-south-1a)</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>payment-processor-partner (Internet)</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Internet Egress Transfer</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F11" s="32" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>1980</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>PCI payment token authorization payloads to payment aggregator</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Optimise payload schema, negotiate AWS Direct Connect / Partner Interconnect</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>Strict PCI DSS network isolation verified</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>DT-PATH-08</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>disbursement-engine (ap-south-1b)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>core-banking-api (eu-west-1 Partner)</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Cross-Region Transfer</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F12" s="33" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Banking settlement synchronization with European partner bank</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>Batch settlement summaries hourly instead of real-time per-transaction RPC</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>GDPR compliance verified; EU data remains strictly within EU boundaries</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>DT-PATH-09</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>staging-environment (ap-south-1)</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>s3-lendflow-dev-temp-dumps (via NAT)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>NAT Gateway Data Processing</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F13" s="32" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>810</v>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Staging regression tests downloading test datasets through NAT Gateway</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>Enable S3 VPC Endpoint on Staging VPC route tables</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>Staging testing unaffected</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>DT-PATH-10</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>monitoring-prometheus (ap-south-1a)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>all-nodes (ap-south-1b, ap-south-1c)</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Cross-AZ Inter-Service Transfer</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F14" s="33" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>640</v>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>Centralised Prometheus scraper pulling metrics across AZ boundaries every 15s</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>Deploy local Prometheus agent per AZ with remote write aggregation</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>Improves monitoring reliability during AZ degradation</t>
+        </is>
+      </c>
+      <c r="K14" s="15" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Top 10 Critical Data Transfer Paths</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="31">
+        <f>SUM(E5:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="18">
+        <f>SUM(G5:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="18">
+        <f>SUM(K5:K14)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day 4: Reserved capacity, savings plans modeling, spot fleet architecture, and sensitivity analysis
</commit_message>
<xml_diff>
--- a/analysis/savings-model.xlsx
+++ b/analysis/savings-model.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Database Analysis" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Storage Analysis" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Data Transfer Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Commitment &amp; Spot" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4639,7 +4640,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -5756,7 +5756,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6337,4 +6336,616 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LendFlow Technologies — Reserved Capacity, Savings Plans &amp; Spot Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Commitment Coverage Gap, Scenario Modeling &amp; Spot Interruption Sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Workload / Instance Family</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Active Fleet Units</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Current On-Demand Spend (USD)</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Current Coverage %</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>1-Yr No Upfront Rate</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>1-Yr Partial Upfront Rate</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>3-Yr Partial Upfront Rate</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Recommended Strategy</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Projected Monthly Savings (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>c5.4xlarge</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Compute Optimized</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>4896</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>3182.4</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>2937.6</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>2448</v>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Right-size first to c5.2xlarge, then cover remaining prod baseline with 1-Yr Partial Upfront CSP</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>1958.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>c5.2xlarge</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Compute Optimized</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>14</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>3427.2</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>2227.68</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>2056.32</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>1713.6</v>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>Cover 8 prod baseline instances with 1-Yr Compute Savings Plan</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>1370.88</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>r5.4xlarge</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Memory Optimized</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>4354.56</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>2830.46</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>2612.74</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>2177.28</v>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Right-size to r5.2xlarge, cover prod DB &amp; Scoring with 1-Yr CSP</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>1741.82</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>r5.2xlarge</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Memory Optimized</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>2903.04</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>1886.98</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>1741.82</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>1451.52</v>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>Cover prod instances with 1-Yr Partial Upfront CSP</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="n">
+        <v>1161.22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>m5.2xlarge</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>General Purpose</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>1658.88</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>1078.27</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>995.33</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>829.4400000000001</v>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>Right-size to m5.xlarge, commit baseline to 1-Yr CSP</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>663.55</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>m5.xlarge</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>General Purpose</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>1105.92</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>718.85</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>663.55</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>552.96</v>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>Cover prod disbursement baseline with 1-Yr CSP</t>
+        </is>
+      </c>
+      <c r="J10" s="15" t="n">
+        <v>442.37</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>db.r5.2xlarge</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>RDS PostgreSQL Multi-AZ</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>2822.4</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>1834.56</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>1693.44</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>1411.2</v>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>1-Yr Partial Upfront RDS Reserved Instance for Primary Prod DB</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>1128.96</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>db.r5.xlarge</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>RDS PostgreSQL Multi-AZ</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>1411.2</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>917.28</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>846.72</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>705.6</v>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>1-Yr Partial Upfront RDS Reserved Instance for Payment Core DB</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>564.48</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>cache.r5.large</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>ElastiCache Redis Cluster</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>1152</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>748.8</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>691.2</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>576</v>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>1-Yr Partial Upfront ElastiCache Reserved Node</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>460.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Commitment Portfolio</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="18">
+        <f>SUM(D5:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>0.0% Baseline</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="17" t="n"/>
+      <c r="I14" s="17" t="n"/>
+      <c r="J14" s="18">
+        <f>SUM(J5:J13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Spot Fleets &amp; Asynchronous Workload Sensitivity Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Workload Pipeline</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Baseline On-Demand Cost</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Spot Discount %</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Net Spot Cost</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Interruption Rate Assumed</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Reprocessing Overhead (USD)</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>Net Monthly Savings (USD)</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>Eligible Instance Alternatives (Min 4 Pools)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>KYC OCR Document Extraction</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>4896</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>1468.8</v>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>54.72</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>3372.48</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>c5.2xlarge, c5a.2xlarge, c6i.2xlarge, m5.2xlarge</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Daily Batch Analytics &amp; ETL</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>2903.04</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>928.97</v>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>1931.97</v>
+      </c>
+      <c r="H20" s="14" t="inlineStr">
+        <is>
+          <t>r5.2xlarge, r5a.2xlarge, r6i.2xlarge, m5.4xlarge</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Credit Risk Simulation Workers</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>595</v>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>1080</v>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>c5.xlarge, c5a.xlarge, c6g.xlarge, m5.xlarge</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>